<commit_message>
doc: add week11 4x step-by-step explain docx files
</commit_message>
<xml_diff>
--- a/docs/岗位/00_EMS_BMS_岗位_优先投递精简版.xlsx
+++ b/docs/岗位/00_EMS_BMS_岗位_优先投递精简版.xlsx
@@ -46,7 +46,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +56,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -85,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -93,6 +105,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -458,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1383,7 +1397,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -1414,7 +1428,7 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；专业厂商/中型平台，匹配度高且竞争相对可控</t>
+          <t>✅ 校招确认！广州储能国企，EMS直接对口，新公司门槛低</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -3327,7 +3341,7 @@
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
@@ -3358,7 +3372,7 @@
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+          <t>✅ 校招确认！七险二金，上海，高度对口，招~30人</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -4651,7 +4665,7 @@
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
@@ -4678,7 +4692,7 @@
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+          <t>⚠️ 硕可投部分副研究员岗，19-30k·15薪</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
@@ -5627,7 +5641,7 @@
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
@@ -5658,7 +5672,7 @@
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；平台好，可作为冲刺投递</t>
+          <t>CATL 2026校招进行中，BMS算法/储能系统开发，20-50w/年</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
@@ -5687,7 +5701,7 @@
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
@@ -5714,7 +5728,7 @@
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；平台好，可作为冲刺投递</t>
+          <t>CATL系子公司，门槛比CATL总部低，校招信息不明确</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
@@ -6326,6 +6340,59 @@
       <c r="N92" s="2" t="inlineStr">
         <is>
           <t>新增候选；需核验校招入口；整合来源：当前主表/优先投递与补充</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>P0 立即优先</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>88</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>较高</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>央企国企优先</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>中国资源循环集团有限公司</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>技术专责/管培生</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>深圳/南京/杭州</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://zgzh.iguopin.com</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>✅ 校招确认！新央企，化学/材料对口，深圳有岗</t>
         </is>
       </c>
     </row>
@@ -8652,7 +8719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8744,130 +8811,138 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>P0 立即优先</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>较高</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>P0 立即优先</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>较高</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>央企国企优先</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>中国三峡新能源(集团)</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>央企/新能源/海上风电/储能(2026校招)</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>武汉/全国</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>www.ctgne.com 校招</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>暂无明显硬伤，仍需核验是否开放</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>武汉补充(央企/半导体)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>广州储能集团有限公司</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>产品研发助理工程师（储能EMS方向）</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>广州</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>手机端 http://bjxapp.cn/t/NjMwODE3OA/</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>✅ 确定有2026校招！2023年成立的新国企，注册资本20亿，广州储能'链主'企业。产品研发岗直接对口EMS项目。新公司校招第一年门槛最低。</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>新公司，薪资待遇待核实</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>✅ 立即投递</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>来源=web-research-2026-07-29；笔记=广州储能集团有明确校招</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>P0 立即优先</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>较高</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>P0 立即优先</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>较高</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>央企国企优先</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>中国中检福建分公司</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>检验检测(电池/新能源)</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>暂无明显硬伤，仍需核验是否开放</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>官网/官方招聘系统核验后投递</t>
-        </is>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>巡检/检测/设备类岗位，按保底稳定线保留；整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/校招可投保底</t>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>中国资源循环集团有限公司</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>技术专责/管培生/工艺工程师（新能源/电池方向）</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>天津（总部）/深圳/南京/杭州</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://zgzh.iguopin.com</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>✅ 确定有2026校招！2025年新央企，国务院国资委直接监管。化学/材料专业在这里是优势不是短板！深圳有子公司。资源循环是政策强推赛道。</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>新央企，业务方向还在搭建中</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>✅ 立即投递</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>来源=web-research-2026-07-29；笔记=中国资环2026校招确认</t>
         </is>
       </c>
     </row>
@@ -8900,16 +8975,24 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>中国华电集团福建分公司</t>
+          <t>中国三峡新能源(集团)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>发电运行/自动化/新能源</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>央企/新能源/海上风电/储能(2026校招)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>武汉/全国</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>www.ctgne.com 校招</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -8922,12 +9005,12 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
+          <t>武汉补充(央企/半导体)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -8960,12 +9043,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>中国华能集团福建分公司</t>
+          <t>中国中检福建分公司</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>发电/新能源</t>
+          <t>检验检测(电池/新能源)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr"/>
@@ -8987,7 +9070,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
+          <t>巡检/检测/设备类岗位，按保底稳定线保留；整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/校招可投保底</t>
         </is>
       </c>
     </row>
@@ -9020,12 +9103,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>中国大唐集团福建分公司</t>
+          <t>中国华电集团福建分公司</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>风光火储/新能源</t>
+          <t>发电运行/自动化/新能源</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -9080,20 +9163,16 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>中国水利电力物资武汉有限公司</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>iguopin.com/官网</t>
-        </is>
-      </c>
+          <t>中国华能集团福建分公司</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>发电/新能源</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9106,12 +9185,12 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
         </is>
       </c>
     </row>
@@ -9144,24 +9223,16 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>中国汽车技术研究中心</t>
+          <t>中国大唐集团福建分公司</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>新能源/算法</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>天津/武汉</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>中汽中心招聘</t>
-        </is>
-      </c>
+          <t>风光火储/新能源</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9174,12 +9245,12 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9283,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>中国电力工程顾问集团中南电力设计院有限公司</t>
+          <t>中国水利电力物资武汉有限公司</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -9276,12 +9347,24 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>中国电建（储能浙江）</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+          <t>中国汽车技术研究中心</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>新能源/算法</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>天津/武汉</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>中汽中心招聘</t>
+        </is>
+      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9294,12 +9377,12 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9332,16 +9415,20 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>中国电气装备集团储能科技</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>EMS软件工程师 | 上海 | 30万/年</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>中国电力工程顾问集团中南电力设计院有限公司</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>武汉</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>iguopin.com/官网</t>
+        </is>
+      </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9354,12 +9441,12 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>原表公司/岗位疑似串位，已自动对调；整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/校招可投保底</t>
+          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9392,20 +9479,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>中国石化集团江汉石油管理局有限公司</t>
+          <t>中国电建（储能浙江）</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>iguopin.com/官网</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9418,12 +9497,12 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部(中石化)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
         </is>
       </c>
     </row>
@@ -9437,7 +9516,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -9456,38 +9535,43 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>中国长安汽车集团/长安新能源体系</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr"/>
+          <t>中国电气装备集团储能科技</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>EMS软件工程师 | 上海 | 30万/年</t>
+        </is>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>重庆/全国/南京等</t>
+          <t>上海（本部）/许昌/天津/济南</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>未找到可引用的具体BMS岗位；官方集团/品牌入口明确</t>
+          <t>campus.51job.com/cnkj2026
+刘老师 021-66698846</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+          <t>✅ 确定有2026校招！招~30人。EMS软件工程师，七险二金，上海落户。储能央企新设，高度对口。</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>暂无明显硬伤，仍需核验是否开放</t>
+          <t>校招已开，抓紧投递。特别优秀可免笔试。</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>查长安招聘官网、深蓝/阿维塔公众号、牛客校招</t>
+          <t>✅ 立即投递</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/优先投递与补充</t>
+          <t>原表公司/岗位疑似串位，已自动对调；整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/校招可投保底</t>
         </is>
       </c>
     </row>
@@ -9520,22 +9604,18 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>中石化工程设计研究院</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>智能低碳研究</t>
-        </is>
-      </c>
+          <t>中国石化集团江汉石油管理局有限公司</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>天津/成都/西安</t>
+          <t>武汉</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>中石化人才招聘网</t>
+          <t>iguopin.com/官网</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -9550,12 +9630,12 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部(中石化)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9588,22 +9668,18 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>中石化石油工程设计</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>智能低碳研究岗</t>
-        </is>
-      </c>
+          <t>中国长安汽车集团/长安新能源体系</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>武汉/成都/西安</t>
+          <t>重庆/全国/南京等</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>中石化人才招聘网</t>
+          <t>未找到可引用的具体BMS岗位；官方集团/品牌入口明确</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -9618,12 +9694,12 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
+          <t>查长安招聘官网、深蓝/阿维塔公众号、牛客校招</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/优先投递与补充</t>
         </is>
       </c>
     </row>
@@ -9656,18 +9732,22 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>中石化石油机械股份有限公司</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>中石化工程设计研究院</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>智能低碳研究</t>
+        </is>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>天津/成都/西安</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>iguopin.com/官网</t>
+          <t>中石化人才招聘网</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -9682,12 +9762,12 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部(中石化)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9720,18 +9800,22 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>中石油深圳新能源研究院</t>
+          <t>中石化石油工程设计</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>储能研发、EMS、BMS、电池/氢能、控制算法、数据分析</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr"/>
+          <t>智能低碳研究岗</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>武汉/成都/西安</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>中石油招聘、国聘网、BOSS、猎聘</t>
+          <t>中石化人才招聘网</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -9746,12 +9830,12 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>查中石油招聘平台/研究院官网/国聘；搜深圳+储能研发</t>
+          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>深圳+央企研发，值得高优先级核验；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/新央企国企重点核验</t>
+          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9784,22 +9868,18 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>中能建储能科技(中储科技)</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>BMS/EMS/PCS储能系统</t>
-        </is>
-      </c>
+          <t>中石化石油机械股份有限公司</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>武汉/福建有协同</t>
+          <t>武汉</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>北极星招聘</t>
+          <t>iguopin.com/官网</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -9814,12 +9894,12 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部(中石化)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9852,18 +9932,18 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>华电华中清洁能源有限公司</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
+          <t>中石油深圳新能源研究院</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>储能研发、EMS、BMS、电池/氢能、控制算法、数据分析</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>iguopin.com/官网</t>
+          <t>中石油招聘、国聘网、BOSS、猎聘</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -9878,12 +9958,12 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>查中石油招聘平台/研究院官网/国聘；搜深圳+储能研发</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>深圳+央企研发，值得高优先级核验；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/新央企国企重点核验</t>
         </is>
       </c>
     </row>
@@ -9916,16 +9996,24 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>华电福新（华电福建）</t>
+          <t>中能建储能科技(中储科技)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>水电/风电/光伏/储能</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+          <t>BMS/EMS/PCS储能系统</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>武汉/福建有协同</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>北极星招聘</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -9938,12 +10026,12 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
+          <t>整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -9976,22 +10064,18 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>南方电网/南网储能/南网科研院</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>储能调度、EMS、自动化控制、电力系统、电化学储能</t>
-        </is>
-      </c>
+          <t>华电华中清洁能源有限公司</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>广东/广西/云南/贵州/海南</t>
+          <t>武汉</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>南方电网官网在线服务区明确有“员工招聘”入口，跳转zhaopin.csg.cn。</t>
+          <t>iguopin.com/官网</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -10006,12 +10090,12 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>直接进南网招聘系统筛“储能/自动化/控制/科研院”。</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>不是新成立，但对口度高，继续保留高优先级。；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/优先投递与补充</t>
+          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -10044,20 +10128,16 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>南方电网储能/南网储能科研院</t>
+          <t>华电福新（华电福建）</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>储能调度、EMS、自动化控制、电化学储能、电力系统</t>
+          <t>水电/风电/光伏/储能</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>南网招聘官网 zhaopin.csg.cn</t>
-        </is>
-      </c>
+      <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10070,12 +10150,12 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>直接进南网招聘系统，按“储能/自动化/控制/科研院”筛选</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>不属于“这两年新成立”，但应保留高优先级投递；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/新央企国企重点核验</t>
+          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
         </is>
       </c>
     </row>
@@ -10108,12 +10188,24 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>南方电网储能科研院</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>南方电网/南网储能/南网科研院</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>储能调度、EMS、自动化控制、电力系统、电化学储能</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>广东/广西/云南/贵州/海南</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>南方电网官网在线服务区明确有“员工招聘”入口，跳转zhaopin.csg.cn。</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10126,12 +10218,12 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>直接进南网招聘系统筛“储能/自动化/控制/科研院”。</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
+          <t>不是新成立，但对口度高，继续保留高优先级。；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/优先投递与补充</t>
         </is>
       </c>
     </row>
@@ -10164,16 +10256,20 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>厦门钨业(省冶金控股)</t>
+          <t>南方电网储能/南网储能科研院</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>新能源材料/BMS</t>
+          <t>储能调度、EMS、自动化控制、电化学储能、电力系统</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>南网招聘官网 zhaopin.csg.cn</t>
+        </is>
+      </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10186,12 +10282,12 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>直接进南网招聘系统，按“储能/自动化/控制/科研院”筛选</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
+          <t>不属于“这两年新成立”，但应保留高优先级投递；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/新央企国企重点核验</t>
         </is>
       </c>
     </row>
@@ -10224,20 +10320,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>国家电力投资集团有限公司湖北分公司</t>
+          <t>南方电网储能科研院</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>iguopin.com/官网</t>
-        </is>
-      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10250,12 +10338,12 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部(国电投)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>适合技术/科研/稳定路线；重点看是否接收应届硕士。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
         </is>
       </c>
     </row>
@@ -10288,12 +10376,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>国家电投福建电力</t>
+          <t>厦门钨业(省冶金控股)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>核能/储能/综合智慧能源</t>
+          <t>新能源材料/BMS</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -10348,7 +10436,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>国家电网公司华中分部</t>
+          <t>国家电力投资集团有限公司湖北分公司</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -10379,7 +10467,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部(国家电网)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部(国电投)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -10412,12 +10500,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>国家能源集团福建公司</t>
+          <t>国家电投福建电力</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>集控/热工/新能源/人工智能</t>
+          <t>核能/储能/综合智慧能源</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -10472,7 +10560,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>国电湖北电力有限公司（国电长源电力股份有限公司）</t>
+          <t>国家电网公司华中分部</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -10536,20 +10624,16 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>大唐湖北能源开发有限公司</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>iguopin.com/官网</t>
-        </is>
-      </c>
+          <t>国家能源集团福建公司</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>集控/热工/新能源/人工智能</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10562,12 +10646,12 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部(大唐)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>整合来源：EMS_BMS_岗位_校招可投版_2026-06-29.xlsx/已剔除_不适合校招</t>
         </is>
       </c>
     </row>
@@ -10600,12 +10684,20 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>广东储能产业发展</t>
+          <t>国电湖北电力有限公司（国电长源电力股份有限公司）</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>武汉</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>iguopin.com/官网</t>
+        </is>
+      </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10618,12 +10710,12 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>先核验是否已有正式校招/社招入口，再决定是否投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部(国家电网)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -10656,12 +10748,20 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>广东新型储能国家研究院</t>
+          <t>大唐湖北能源开发有限公司</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>武汉</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>iguopin.com/官网</t>
+        </is>
+      </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10674,12 +10774,12 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>先核验是否已有正式校招/社招入口，再决定是否投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部(大唐)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -10712,20 +10812,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>武汉建筑材料工业设计研究院有限公司</t>
+          <t>广东储能产业发展</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>iguopin.com/官网</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
@@ -10738,12 +10830,12 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>官网/官方招聘系统核验后投递</t>
         </is>
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>先核验是否已有正式校招/社招入口，再决定是否投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
         </is>
       </c>
     </row>
@@ -10757,7 +10849,7 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
@@ -10776,23 +10868,19 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>武汉普天电源有限公司</t>
+          <t>广东新型储能国家研究院</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>武汉</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>iguopin.com/官网</t>
+          <t>zhaopin@naesic.com</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+          <t>⚠️ 以博士/博士后为主，硕士可投部分副研究员岗(19-30k·15薪)。门槛高但薪资诱人。</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -10802,12 +10890,12 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>⚠️ 冲刺项，硕可试</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>先核验是否已有正式校招/社招入口，再决定是否投递。；整合来源：EMS_BMS_央企国企_四省全量_20260629.xlsx/四省央企国企</t>
         </is>
       </c>
     </row>
@@ -10840,22 +10928,18 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>深南电(储能EMS)</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>储能EMS专业工程师(国企背景)</t>
-        </is>
-      </c>
+          <t>武汉建筑材料工业设计研究院有限公司</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>深圳</t>
+          <t>武汉</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>北极星储能招聘</t>
+          <t>iguopin.com/官网</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -10870,12 +10954,12 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>深圳新增(储能/BMS)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -10908,7 +10992,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>湖北三江航天江河化工科技有限公司</t>
+          <t>武汉普天电源有限公司</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
@@ -10972,18 +11056,22 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>湖北省电力装备有限公司</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr"/>
+          <t>深南电(储能EMS)</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>储能EMS专业工程师(国企背景)</t>
+        </is>
+      </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>武汉</t>
+          <t>深圳</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>iguopin.com/官网</t>
+          <t>北极星储能招聘</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -10998,12 +11086,12 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+          <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
         </is>
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+          <t>深圳新增(储能/BMS)；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
       </c>
     </row>
@@ -11036,7 +11124,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>湖北龙源新能源有限公司</t>
+          <t>湖北三江航天江河化工科技有限公司</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
@@ -11100,40 +11188,168 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
+          <t>湖北省电力装备有限公司</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>武汉</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>iguopin.com/官网</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>暂无明显硬伤，仍需核验是否开放</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>P0 立即优先</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>较高</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>央企国企优先</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>湖北龙源新能源有限公司</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>武汉</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>iguopin.com/官网</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>暂无明显硬伤，仍需核验是否开放</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>央企在鄂分部/二级公司，武汉本地，稳定待遇</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>湖北省93家央企国企清单-央企分部；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>P0 立即优先</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>较高</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>央企国企优先</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
           <t>福建省工业控股集团</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>工业/制造业/投资</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>福州</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>官网</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；央国企省公司/子公司/能源平台，稳定且专业可解释</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>暂无明显硬伤，仍需核验是否开放</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>暂无明显硬伤，仍需核验是否开放</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>稳定路线；优先官网/国聘/集团校招平台核验并投递。</t>
         </is>
       </c>
-      <c r="N39" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>福建省央国企；省属国企，待确认新能源业务；福建省央国企；整合来源：EMS_BMS_岗位_四表精简版_重点核验合并版_backup_before_docx补充_2026-07-27.xlsx/央企国企</t>
         </is>
@@ -11716,7 +11932,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -11744,10 +11960,15 @@
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Talent.CATL.com
+catl-campus@catl.com</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；平台好，可作为冲刺投递</t>
+          <t>CATL 2026校招进行中！BMS软件与算法/储能系统开发岗，20-50w/年。专业门槛仍在，但今年明确写了化学/材料可投。</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -11757,7 +11978,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>官网/官方招聘系统核验后投递</t>
+          <t>可投，别抱太大期望</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -11776,7 +11997,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -11803,7 +12024,7 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；平台好，可作为冲刺投递</t>
+          <t>CATL系独立储能子公司，门槛比CATL总部低。但校招信息不明确，需关注。</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -13843,7 +14064,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -13874,7 +14095,7 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>EMS/BMS/储能/电池管理方向强匹配；化学/材料背景容易讲通；地点符合南方/重点城市偏好；专业厂商/中型平台，匹配度高且竞争相对可控</t>
+          <t>✅ 校招确认！广州储能国企，EMS直接对口</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">

</xml_diff>